<commit_message>
tambah kolom standar BBM tiap merk tiap jenis alat berat, update dashboard menambahkan persentase unit yg masuk analisa dan tidak
</commit_message>
<xml_diff>
--- a/Database_Jarak_Pabrik.xlsx
+++ b/Database_Jarak_Pabrik.xlsx
@@ -1517,7 +1517,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>13.5076</v>
+        <v>12.6777</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>13.5076</v>
+        <v>12.6777</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>13.5076</v>
+        <v>12.6777</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -2317,16 +2317,16 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>377.8862</v>
+        <v>40.7071</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Sukses (Kecamatan OSM)</t>
+          <t>Sukses (Kota/Kab OSM)</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Kec. Gresik, Kabupaten Gresik, Jawa Timur</t>
+          <t>Kabupaten Gresik, Jawa Timur</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2377,7 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>13.5411</v>
+        <v>12.9025</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
@@ -2977,16 +2977,16 @@
         </is>
       </c>
       <c r="B128" t="n">
-        <v>377.8862</v>
+        <v>40.7071</v>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Sukses (Kecamatan OSM)</t>
+          <t>Sukses (Kota/Kab OSM)</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Kec. Gresik, Kabupaten Gresik, Jawa Timur</t>
+          <t>Kabupaten Gresik, Jawa Timur</t>
         </is>
       </c>
     </row>
@@ -3337,16 +3337,16 @@
         </is>
       </c>
       <c r="B146" t="n">
-        <v>377.8862</v>
+        <v>40.7071</v>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Sukses (Kecamatan OSM)</t>
+          <t>Sukses (Kota/Kab OSM)</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Kec. Gresik, Kabupaten Gresik, Jawa Timur</t>
+          <t>Kabupaten Gresik, Jawa Timur</t>
         </is>
       </c>
     </row>

</xml_diff>